<commit_message>
Use existing Modashop swimwear category
</commit_message>
<xml_diff>
--- a/templates/export-template.xlsx
+++ b/templates/export-template.xlsx
@@ -1070,7 +1070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1152,53 +1152,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>85901631</v>
+        <v>31935910</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Женщинам</t>
+          <t>Купальники</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Жінкам</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>85901740</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Одежда</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Одяг</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>85901631</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>85929329</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
           <t>Купальники</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Купальники</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>85901740</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>31935910</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[codex] Require manual import price and use Modashop swimwear category (#2)
* feat: require manual import price

* docs: document cleaning ui outputs

* Use existing Modashop swimwear category
</commit_message>
<xml_diff>
--- a/templates/export-template.xlsx
+++ b/templates/export-template.xlsx
@@ -1070,7 +1070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1152,53 +1152,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>85901631</v>
+        <v>31935910</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Женщинам</t>
+          <t>Купальники</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Жінкам</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>85901740</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Одежда</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Одяг</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>85901631</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>85929329</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
           <t>Купальники</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Купальники</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>85901740</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>31935910</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>